<commit_message>
Add pepline line_deconv scripts and data
Introduce pepline line deconvolution tooling and results. Added pepline/line_deconv.py, a test notebook, and several result spreadsheets; updated pepline annotation.py, deconv_dataframe.py, and line_finding.py; added/updated sample deconvolution data under data/short_peptide (including charged_annotated and charged_replaced files) and replaced annotated outputs. Removed a temporary long_peptide workbook and updated various .DS_Store and annot.xlsx files. This brings initial processing, line-finding and deconvolution outputs into the repository for further development and testing.
</commit_message>
<xml_diff>
--- a/pepline/annot.xlsx
+++ b/pepline/annot.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="z7_611_dm2_NCE25" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VEA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4+" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -1848,7 +1849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1864,7 +1865,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>All Coverage=93.3%</t>
+          <t>All Coverage=100.0%</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1893,14 +1894,20 @@
         </is>
       </c>
       <c r="I1" s="1" t="n">
-        <v>-229.111</v>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+        <v>-654.838</v>
+      </c>
+      <c r="J1" s="1" t="n">
+        <v>-229.112</v>
+      </c>
+      <c r="K1" s="1" t="n">
+        <v>-100.069</v>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Row Count</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>theoretical mass</t>
         </is>
@@ -1915,6 +1922,967 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>V</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>+*</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>(100.076, 1507.786)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>b2, y13</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>+*</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>(229.118, 1378.744)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>b3, y12</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0, (+1)-654.838, [1.0, 1.0], (0.001, 0.003), [3]</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0, (+1)-229.112, [1.0, 1.0], (0.001, 0.004), [329] ('used')</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>(300.155, 1307.707)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>b4, y11</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0, 0, [1.0, 2.0], (0.002, 0.004), [9]</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>(415.182, 1192.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>b5, y10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0, 0, [1.0, 2.0], (0.002, 0.003), [12]</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.001, 0.006), [329] ('used')</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>(0)-100.069, 0, [1.0, 2.0], (0.018, 0.003), [28]</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>(528.266, 1079.596)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>b6, y9</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0, 0, [1.0, 2.0], (0.002, 0.003), [10]</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.001, 0.005), [7]</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>(+1)-100.069, 0, [1.0, 1.0], (0.001, 0.005), [46]</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>(599.303, 1008.558)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>b7, y8</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.001, 0.005), [19]</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>(656.325, 951.537)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>b8, y7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 1.0], (0.002, 0.004), [24]</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.0, 0.004), [2]</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>(+1)-100.069, 0, [1.0, 1.0], (0.001, 0.004), [23]</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>3</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>(793.384, 814.478)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>b9, y6</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 1.0], (0.002, 0.003), [36]</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.0, 0.003), [11]</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>(850.405, 757.457)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>b10, y5</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 1.0], (0.002, 0.003), [18]</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.001, 0.003), [5]</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>(978.464, 629.398)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>b11, y4</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 1.0], (0.003, 0.002), [34]</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.002, 0.002), [4]</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>0, (+1)-100.069, [1.0, 1.0], (0.006, 0.001), [29] ('used')</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>3</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>(1107.506, 500.355)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>b12, y3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 1.0], (0.003, 0.002), [61]</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.003, 0.002), [13]</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>(+1)-100.069, 0, [1.0, 1.0], (0.003, 0.002), [29] ('used')</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>3</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>(1206.575, 401.287)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>b13, y2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.004, 0.001), [14]</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>(1319.659, 288.203)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>b14, y1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>(+1)-229.112, 0, [1.0, 1.0], (0.005, 0.001), [1]</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>(1432.743, 175.119)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Col Count</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>11</v>
+      </c>
+      <c r="K16" t="n">
+        <v>5</v>
+      </c>
+      <c r="L16" t="n">
+        <v>14</v>
+      </c>
+      <c r="M16" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>FFC</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>44</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>12</v>
+      </c>
+      <c r="J17" t="n">
+        <v>40</v>
+      </c>
+      <c r="K17" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>FPR0</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>FPR1</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>b2</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>b1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>FPR0_LIST_1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>(603.7931, 175.1196, [1.0, 2.0], 70.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>FPR0_LIST_2</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>(175.1196, 603.7931, [2.0, 1.0], 70.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>FPR0_LIST_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>TFPR0_LIST_1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>(603.7931, 350.2392, 954.0323)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>TFPR0_LIST_2</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>(350.2392, 603.7931, 954.0323)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>TFPR0_LIST_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>FPR1_LIST_1</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>(+3)-102.076, ???, [1.0, 2.0], (0.002, 'n/a'), [67]| ('used')</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>FPR1_LIST_2</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>(+2)-101.072, ???, [1.0, 2.0], (0.002, 'n/a'), [67]| ('used')</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>FPR1_LIST_3</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>(+1)-100.069, ???, [1.0, 2.0], (0.002, 'n/a'), [67]| ('used')</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>TFPR1_LIST_1</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>(201.0877, 1307.7502, 1508.8379)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>TFPR1_LIST_2</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>(201.0877, 1307.7502, 1508.8379)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>TFPR1_LIST_3</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>(201.0877, 1307.7502, 1508.8379)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>Modifications_Count</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" t="n">
+        <v>5</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>|SIM(A*,B)|</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>8</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>7</v>
+      </c>
+      <c r="K34" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>|DIFF(A*,B)|</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" t="n">
+        <v>4</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>N=1000</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>All Coverage=72.7%</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>isocolumn:0</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>parent(0.02)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>1(0.05)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>2(0.03)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>3(0.04)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>4(0.06)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Row Count</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>theoretical mass</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>b1, y32</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>H</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1933,55 +2901,63 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>(100.076, 1507.786)</t>
+          <t>(138.066, 3627.763)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>b2, y13</t>
+          <t>b2, y31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>+*</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0, 0, [1.0, 3.0], (0.001, 0.018), [167]</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>(229.118, 1378.744)</t>
+          <t>(209.103, 3556.726)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>b3, y12</t>
+          <t>b3, y30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>+</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -1989,34 +2965,30 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0, (+1)-229.111, [1.0, 1.0], (0.001, 0.003), [329] ('used')</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>(300.155, 1307.707)</t>
+          <t>(324.13, 3441.699)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>b4, y11</t>
+          <t>b4, y29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>+</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -2024,34 +2996,30 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.003, 0.004), [48]</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>(415.182, 1192.68)</t>
+          <t>(381.152, 3384.678)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>b5, y10</t>
+          <t>b5, y28</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>+</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -2059,77 +3027,61 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.002, 0.006), [329] ('used')</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>(528.266, 1079.596)</t>
+          <t>(468.184, 3297.646)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>b6, y9</t>
+          <t>b6, y27</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>(0, 0)</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>0, 0, [2.0, 1.0], (0.001, 0.005), [45]</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.002, 0.005), [7]</t>
-        </is>
-      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>(599.303, 1008.558)</t>
+          <t>(615.252, 3150.578)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>b7, y8</t>
+          <t>b7, y26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>+</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -2137,72 +3089,56 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.002, 0.005), [19]</t>
-        </is>
-      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>(656.325, 951.537)</t>
+          <t>(702.284, 3063.545)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>b8, y7</t>
+          <t>b8, y25</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>(0, 0)</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>0, 0, [2.0, 1.0], (0.002, 0.004), [24]</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.001, 0.004), [2]</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>(793.384, 814.478)</t>
+          <t>(817.311, 2948.519)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>b9, y6</t>
+          <t>b9, y24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2217,35 +3153,31 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0, 0, [2.0, 1.0], (0.002, 0.003), [36]</t>
+          <t>0, 0, [2.0, 2.0], (0.004, 0.017), [216]</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.001, 0.003), [11]</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>(850.405, 757.457)</t>
+          <t>(946.354, 2819.476)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>b10, y5</t>
+          <t>b10, y23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2260,35 +3192,31 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0, 0, [2.0, 1.0], (0.002, 0.003), [18]</t>
+          <t>0, 0, [2.0, 2.0], (0.005, 0.017), [93]</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.0, 0.003), [5]</t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>(978.464, 629.398)</t>
+          <t>(1077.394, 2688.435)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>b11, y4</t>
+          <t>b11, y22</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>N</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2296,34 +3224,38 @@
           <t>+</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.005, 0.016), [80]</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.001, 0.002), [4]</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="n">
         <v>1</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>(1107.506, 500.355)</t>
+          <t>(1191.437, 2574.393)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>b12, y3</t>
+          <t>b12, y21</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2338,35 +3270,31 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0, 0, [2.0, 1.0], (0.003, 0.002), [61]</t>
+          <t>0, 0, [2.0, 2.0], (0.006, 0.014), [11]</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.002, 0.002), [13]</t>
-        </is>
-      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>(1206.575, 401.287)</t>
+          <t>(1292.485, 2473.345)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>b13, y2</t>
+          <t>b13, y20</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2374,34 +3302,38 @@
           <t>+</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.006, 0.014), [17]</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.003, 0.001), [14]</t>
-        </is>
-      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="n">
         <v>1</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>(1319.659, 288.203)</t>
+          <t>(1405.569, 2360.261)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>b14, y1</t>
+          <t>b14, y19</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2409,34 +3341,38 @@
           <t>+</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.007, 0.013), [19]</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>(+1)-229.111, 0, [1.0, 1.0], (0.004, 0.001), [1]</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="n">
         <v>1</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>(1432.743, 175.119)</t>
+          <t>(1518.653, 2247.177)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Col Count</t>
+          <t>b15, y18</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2444,423 +3380,1117 @@
           <t>+</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="n">
-        <v>5</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>12</v>
-      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.008, 0.013), [135]</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
-        <v>14</v>
-      </c>
-      <c r="K16" t="n">
-        <v>14</v>
+        <v>1</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>(1633.68, 2132.15)</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>FFC</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+          <t>b16, y17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="n">
-        <v>20</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>44</v>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>(1747.723, 2018.107)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>FPR0</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+          <t>b17, y16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.009, 0.01), [42]</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>(1860.807, 1905.023)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>FPR1</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+          <t>b18, y15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.01, 0.01), [49]</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>(1931.844, 1833.986)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>offset</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+          <t>b19, y14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.011, 0.008), [78]</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>b2</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>(2002.881, 1762.949)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>FPR0_LIST_1</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+          <t>b20, y13</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.014, 0.007), [226]</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>(2158.982, 1606.847)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>FPR0_LIST_2</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+          <t>b21, y12</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.014, 0.007), [236]</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>(2274.009, 1491.821)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>FPR0_LIST_3</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+          <t>b22, y11</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.014, 0.006), [164]</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>(2421.077, 1344.752)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>TFPR0_LIST_1</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+          <t>b23, y10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.016, 0.005), [25]</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>(2534.162, 1231.668)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>TFPR0_LIST_2</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+          <t>b24, y9</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.017, 0.005), [54]</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>(2648.204, 1117.625)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>TFPR0_LIST_3</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+          <t>b25, y8</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>0, 0, [2.0, 2.0], (0.019, 0.004), [107]</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>(2834.284, 931.546)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>FPR1_LIST_1</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+          <t>b26, y7</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>0, 0, [3.0, 1.0], (0.014, 0.005), [6]</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>(2947.368, 818.462)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>FPR1_LIST_2</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+          <t>b27, y6</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0, 0, [3.0, 1.0], (0.015, 0.004), [4]</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>(3060.452, 705.378)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>FPR1_LIST_3</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
+          <t>b28, y5</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>0, 0, [3.0, 1.0], (0.016, 0.003), [24]</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>+1, 0, [3.0, 1.0], (0.015, 0.003), [15]</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="J29" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>(3188.511, 577.319)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>TFPR1_LIST_1</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
+          <t>b29, y4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>0, 0, [3.0, 1.0], (0.018, 0.003), [1]</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>0, +1, [3.0, 1.0], (0.018, 0.003), [37]</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="J30" t="n">
+        <v>2</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>(3289.558, 476.271)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>TFPR1_LIST_2</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+          <t>b30, y3</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>0, 0, [3.0, 1.0], (0.019, 0.002), [7]</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>0, +1, [3.0, 1.0], (0.019, 0.002), [205]</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="J31" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>(3417.653, 348.176)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>TFPR1_LIST_3</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
+          <t>b31, y2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>(2, 0)</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>+2, 0, [3.0, 1.0], (0.018, 0.001), [31]</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>(3530.737, 235.092)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>Modifications_Count</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0</v>
+          <t>b32, y1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" t="n">
-        <v>2</v>
-      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="n">
         <v>0</v>
       </c>
-      <c r="K33" t="n">
-        <v>0</v>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>(3631.785, 134.045)</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>|SIM(A*,B)|</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
+          <t>Col Count</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>5</v>
-      </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>32</v>
+      </c>
+      <c r="K34" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>|DIFF(A*,B)|</t>
+          <t>FFC</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>207</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>FPR0</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>FPR1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>offset</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>FPR0_LIST_1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>FPR0_LIST_2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>FPR0_LIST_3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>TFPR0_LIST_1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>TFPR0_LIST_2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>TFPR0_LIST_3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>FPR1_LIST_1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>FPR1_LIST_2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>FPR1_LIST_3</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>TFPR1_LIST_1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>TFPR1_LIST_2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>TFPR1_LIST_3</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>Modifications_Count</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>|SIM(A*,B)|</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="n">
+        <v>22</v>
+      </c>
+      <c r="F52" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>|DIFF(A*,B)|</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>